<commit_message>
osphd migration to CCS; age by cause work; other clean up
</commit_message>
<xml_diff>
--- a/myCBD/myInfo/CCS Code and Names Linkage.xlsx
+++ b/myCBD/myInfo/CCS Code and Names Linkage.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="442">
   <si>
     <t>Tuberculosis</t>
   </si>
@@ -1340,10 +1340,7 @@
     <t>ccsName3</t>
   </si>
   <si>
-    <t>birthPregnancyRelated</t>
-  </si>
-  <si>
-    <t>Y</t>
+    <t>birth</t>
   </si>
 </sst>
 </file>
@@ -1431,7 +1428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1444,7 +1441,6 @@
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1749,7 +1745,7 @@
     <col min="6" max="6" width="78.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="141" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="61.5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>435</v>
       </c>
@@ -1791,8 +1787,8 @@
       <c r="F2" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>442</v>
+      <c r="G2" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1814,8 +1810,8 @@
       <c r="F3" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>442</v>
+      <c r="G3" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1837,8 +1833,8 @@
       <c r="F4" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>442</v>
+      <c r="G4" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1860,8 +1856,8 @@
       <c r="F5" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>442</v>
+      <c r="G5" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1883,8 +1879,8 @@
       <c r="F6" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>442</v>
+      <c r="G6" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1906,8 +1902,8 @@
       <c r="F7" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>442</v>
+      <c r="G7" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1929,8 +1925,8 @@
       <c r="F8" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>442</v>
+      <c r="G8" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1952,8 +1948,8 @@
       <c r="F9" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>442</v>
+      <c r="G9" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1975,8 +1971,8 @@
       <c r="F10" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>442</v>
+      <c r="G10" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1998,8 +1994,8 @@
       <c r="F11" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>442</v>
+      <c r="G11" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -2021,8 +2017,8 @@
       <c r="F12" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>442</v>
+      <c r="G12" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -2044,8 +2040,8 @@
       <c r="F13" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>442</v>
+      <c r="G13" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -2067,8 +2063,8 @@
       <c r="F14" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>442</v>
+      <c r="G14" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -2090,8 +2086,8 @@
       <c r="F15" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="G15" s="5" t="s">
-        <v>442</v>
+      <c r="G15" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -2113,8 +2109,8 @@
       <c r="F16" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G16" s="5" t="s">
-        <v>442</v>
+      <c r="G16" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2136,8 +2132,8 @@
       <c r="F17" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G17" s="5" t="s">
-        <v>442</v>
+      <c r="G17" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -2159,8 +2155,8 @@
       <c r="F18" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>442</v>
+      <c r="G18" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2182,8 +2178,8 @@
       <c r="F19" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="G19" s="5" t="s">
-        <v>442</v>
+      <c r="G19" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2205,8 +2201,8 @@
       <c r="F20" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>442</v>
+      <c r="G20" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -2228,8 +2224,8 @@
       <c r="F21" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="G21" s="5" t="s">
-        <v>442</v>
+      <c r="G21" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -2251,8 +2247,8 @@
       <c r="F22" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>442</v>
+      <c r="G22" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -2274,8 +2270,8 @@
       <c r="F23" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>442</v>
+      <c r="G23" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2297,8 +2293,8 @@
       <c r="F24" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="G24" s="5" t="s">
-        <v>442</v>
+      <c r="G24" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2320,8 +2316,8 @@
       <c r="F25" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G25" s="5" t="s">
-        <v>442</v>
+      <c r="G25" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -2343,8 +2339,8 @@
       <c r="F26" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="G26" s="5" t="s">
-        <v>442</v>
+      <c r="G26" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -2366,8 +2362,8 @@
       <c r="F27" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G27" s="5" t="s">
-        <v>442</v>
+      <c r="G27" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -2389,8 +2385,8 @@
       <c r="F28" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G28" s="5" t="s">
-        <v>442</v>
+      <c r="G28" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -2412,8 +2408,8 @@
       <c r="F29" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="G29" s="5" t="s">
-        <v>442</v>
+      <c r="G29" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -2435,6 +2431,9 @@
       <c r="F30" s="2" t="s">
         <v>307</v>
       </c>
+      <c r="G30" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
@@ -2455,6 +2454,9 @@
       <c r="F31" s="2" t="s">
         <v>309</v>
       </c>
+      <c r="G31" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
@@ -2475,8 +2477,11 @@
       <c r="F32" s="2" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>216</v>
       </c>
@@ -2495,8 +2500,11 @@
       <c r="F33" s="2" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>217</v>
       </c>
@@ -2515,8 +2523,11 @@
       <c r="F34" s="2" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>60</v>
       </c>
@@ -2535,8 +2546,11 @@
       <c r="F35" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>62</v>
       </c>
@@ -2555,8 +2569,11 @@
       <c r="F36" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>59</v>
       </c>
@@ -2575,8 +2592,11 @@
       <c r="F37" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>63</v>
       </c>
@@ -2595,8 +2615,11 @@
       <c r="F38" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>64</v>
       </c>
@@ -2615,8 +2638,11 @@
       <c r="F39" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>61</v>
       </c>
@@ -2635,8 +2661,11 @@
       <c r="F40" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>109</v>
       </c>
@@ -2655,8 +2684,11 @@
       <c r="F41" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>100</v>
       </c>
@@ -2675,8 +2707,11 @@
       <c r="F42" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>116</v>
       </c>
@@ -2695,8 +2730,11 @@
       <c r="F43" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>115</v>
       </c>
@@ -2715,8 +2753,11 @@
       <c r="F44" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>107</v>
       </c>
@@ -2735,8 +2776,11 @@
       <c r="F45" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>106</v>
       </c>
@@ -2755,8 +2799,11 @@
       <c r="F46" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>105</v>
       </c>
@@ -2775,8 +2822,11 @@
       <c r="F47" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>108</v>
       </c>
@@ -2795,8 +2845,11 @@
       <c r="F48" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>101</v>
       </c>
@@ -2815,8 +2868,11 @@
       <c r="F49" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>98</v>
       </c>
@@ -2835,8 +2891,11 @@
       <c r="F50" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>96</v>
       </c>
@@ -2855,8 +2914,11 @@
       <c r="F51" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>120</v>
       </c>
@@ -2875,8 +2937,11 @@
       <c r="F52" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>99</v>
       </c>
@@ -2895,8 +2960,11 @@
       <c r="F53" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>113</v>
       </c>
@@ -2915,8 +2983,11 @@
       <c r="F54" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>102</v>
       </c>
@@ -2935,8 +3006,11 @@
       <c r="F55" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G55" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>110</v>
       </c>
@@ -2955,8 +3029,11 @@
       <c r="F56" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G56" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>111</v>
       </c>
@@ -2975,8 +3052,11 @@
       <c r="F57" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G57" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>104</v>
       </c>
@@ -2995,8 +3075,11 @@
       <c r="F58" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G58" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>117</v>
       </c>
@@ -3015,8 +3098,11 @@
       <c r="F59" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G59" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>121</v>
       </c>
@@ -3035,8 +3121,11 @@
       <c r="F60" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G60" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>97</v>
       </c>
@@ -3055,8 +3144,11 @@
       <c r="F61" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G61" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>114</v>
       </c>
@@ -3075,8 +3167,11 @@
       <c r="F62" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G62" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>118</v>
       </c>
@@ -3095,8 +3190,11 @@
       <c r="F63" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G63" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>103</v>
       </c>
@@ -3115,8 +3213,11 @@
       <c r="F64" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G64" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>112</v>
       </c>
@@ -3135,8 +3236,11 @@
       <c r="F65" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G65" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>119</v>
       </c>
@@ -3155,8 +3259,11 @@
       <c r="F66" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G66" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>143</v>
       </c>
@@ -3175,8 +3282,11 @@
       <c r="F67" s="2" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>147</v>
       </c>
@@ -3195,8 +3305,11 @@
       <c r="F68" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G68" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>142</v>
       </c>
@@ -3215,8 +3328,11 @@
       <c r="F69" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G69" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>149</v>
       </c>
@@ -3235,8 +3351,11 @@
       <c r="F70" s="2" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G70" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>137</v>
       </c>
@@ -3255,8 +3374,11 @@
       <c r="F71" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G71" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>136</v>
       </c>
@@ -3275,8 +3397,11 @@
       <c r="F72" s="2" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G72" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>146</v>
       </c>
@@ -3295,8 +3420,11 @@
       <c r="F73" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G73" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>138</v>
       </c>
@@ -3315,8 +3443,11 @@
       <c r="F74" s="2" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G74" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>140</v>
       </c>
@@ -3335,8 +3466,11 @@
       <c r="F75" s="2" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G75" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>139</v>
       </c>
@@ -3355,8 +3489,11 @@
       <c r="F76" s="2" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G76" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>153</v>
       </c>
@@ -3375,8 +3512,11 @@
       <c r="F77" s="2" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G77" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>135</v>
       </c>
@@ -3395,8 +3535,11 @@
       <c r="F78" s="2" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G78" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>145</v>
       </c>
@@ -3415,8 +3558,11 @@
       <c r="F79" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G79" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>154</v>
       </c>
@@ -3435,8 +3581,11 @@
       <c r="F80" s="2" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G80" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>141</v>
       </c>
@@ -3455,8 +3604,11 @@
       <c r="F81" s="2" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G81" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>155</v>
       </c>
@@ -3475,8 +3627,11 @@
       <c r="F82" s="2" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G82" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>151</v>
       </c>
@@ -3495,8 +3650,11 @@
       <c r="F83" s="2" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G83" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>152</v>
       </c>
@@ -3515,8 +3673,11 @@
       <c r="F84" s="2" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G84" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>148</v>
       </c>
@@ -3535,8 +3696,11 @@
       <c r="F85" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G85" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>144</v>
       </c>
@@ -3555,8 +3719,11 @@
       <c r="F86" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G86" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>157</v>
       </c>
@@ -3575,8 +3742,11 @@
       <c r="F87" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G87" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>160</v>
       </c>
@@ -3595,8 +3765,11 @@
       <c r="F88" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G88" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>158</v>
       </c>
@@ -3615,8 +3788,11 @@
       <c r="F89" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G89" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>169</v>
       </c>
@@ -3635,8 +3811,11 @@
       <c r="F90" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G90" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>174</v>
       </c>
@@ -3655,8 +3834,11 @@
       <c r="F91" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G91" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>163</v>
       </c>
@@ -3675,8 +3857,11 @@
       <c r="F92" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G92" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>164</v>
       </c>
@@ -3695,8 +3880,11 @@
       <c r="F93" s="2" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G93" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>165</v>
       </c>
@@ -3715,8 +3903,11 @@
       <c r="F94" s="2" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G94" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>168</v>
       </c>
@@ -3735,8 +3926,11 @@
       <c r="F95" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G95" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>173</v>
       </c>
@@ -3755,8 +3949,11 @@
       <c r="F96" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G96" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>171</v>
       </c>
@@ -3775,8 +3972,11 @@
       <c r="F97" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G97" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>156</v>
       </c>
@@ -3795,8 +3995,11 @@
       <c r="F98" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G98" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>167</v>
       </c>
@@ -3815,8 +4018,11 @@
       <c r="F99" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G99" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>162</v>
       </c>
@@ -3835,8 +4041,11 @@
       <c r="F100" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G100" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>161</v>
       </c>
@@ -3855,8 +4064,11 @@
       <c r="F101" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G101" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>175</v>
       </c>
@@ -3875,8 +4087,11 @@
       <c r="F102" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G102" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>166</v>
       </c>
@@ -3895,8 +4110,11 @@
       <c r="F103" s="2" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G103" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>172</v>
       </c>
@@ -3915,8 +4133,11 @@
       <c r="F104" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G104" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>170</v>
       </c>
@@ -3935,8 +4156,11 @@
       <c r="F105" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G105" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>159</v>
       </c>
@@ -3955,8 +4179,11 @@
       <c r="F106" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G106" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>208</v>
       </c>
@@ -3975,8 +4202,11 @@
       <c r="F107" s="2" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G107" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>201</v>
       </c>
@@ -3995,8 +4225,11 @@
       <c r="F108" s="2" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G108" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>203</v>
       </c>
@@ -4015,8 +4248,11 @@
       <c r="F109" s="2" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G109" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>206</v>
       </c>
@@ -4035,8 +4271,11 @@
       <c r="F110" s="2" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G110" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>209</v>
       </c>
@@ -4055,8 +4294,11 @@
       <c r="F111" s="2" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G111" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>212</v>
       </c>
@@ -4075,8 +4317,11 @@
       <c r="F112" s="2" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G112" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>211</v>
       </c>
@@ -4095,8 +4340,11 @@
       <c r="F113" s="2" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G113" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>204</v>
       </c>
@@ -4115,8 +4363,11 @@
       <c r="F114" s="2" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G114" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>207</v>
       </c>
@@ -4135,8 +4386,11 @@
       <c r="F115" s="2" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G115" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>202</v>
       </c>
@@ -4155,8 +4409,11 @@
       <c r="F116" s="2" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G116" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>205</v>
       </c>
@@ -4175,8 +4432,11 @@
       <c r="F117" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G117" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>210</v>
       </c>
@@ -4195,8 +4455,11 @@
       <c r="F118" s="2" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G118" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>89</v>
       </c>
@@ -4215,8 +4478,11 @@
       <c r="F119" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G119" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>86</v>
       </c>
@@ -4235,8 +4501,11 @@
       <c r="F120" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G120" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>85</v>
       </c>
@@ -4255,8 +4524,11 @@
       <c r="F121" s="2" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G121" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>93</v>
       </c>
@@ -4275,8 +4547,11 @@
       <c r="F122" s="2" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G122" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>77</v>
       </c>
@@ -4295,8 +4570,11 @@
       <c r="F123" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G123" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>83</v>
       </c>
@@ -4315,8 +4593,11 @@
       <c r="F124" s="2" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G124" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>88</v>
       </c>
@@ -4335,8 +4616,11 @@
       <c r="F125" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G125" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>84</v>
       </c>
@@ -4355,8 +4639,11 @@
       <c r="F126" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G126" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>90</v>
       </c>
@@ -4375,8 +4662,11 @@
       <c r="F127" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G127" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>76</v>
       </c>
@@ -4395,8 +4685,11 @@
       <c r="F128" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G128" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>80</v>
       </c>
@@ -4415,8 +4708,11 @@
       <c r="F129" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G129" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>78</v>
       </c>
@@ -4435,8 +4731,11 @@
       <c r="F130" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G130" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>94</v>
       </c>
@@ -4455,8 +4754,11 @@
       <c r="F131" s="2" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G131" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>91</v>
       </c>
@@ -4475,8 +4777,11 @@
       <c r="F132" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G132" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>81</v>
       </c>
@@ -4495,8 +4800,11 @@
       <c r="F133" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G133" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>95</v>
       </c>
@@ -4515,8 +4823,11 @@
       <c r="F134" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G134" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>92</v>
       </c>
@@ -4535,8 +4846,11 @@
       <c r="F135" s="2" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G135" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>82</v>
       </c>
@@ -4555,8 +4869,11 @@
       <c r="F136" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G136" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>79</v>
       </c>
@@ -4575,8 +4892,11 @@
       <c r="F137" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G137" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>87</v>
       </c>
@@ -4595,8 +4915,11 @@
       <c r="F138" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G138" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>124</v>
       </c>
@@ -4615,8 +4938,11 @@
       <c r="F139" s="2" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G139" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>125</v>
       </c>
@@ -4635,8 +4961,11 @@
       <c r="F140" s="2" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G140" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>129</v>
       </c>
@@ -4655,8 +4984,11 @@
       <c r="F141" s="2" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G141" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>128</v>
       </c>
@@ -4675,8 +5007,11 @@
       <c r="F142" s="2" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G142" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>127</v>
       </c>
@@ -4695,8 +5030,11 @@
       <c r="F143" s="2" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G143" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>123</v>
       </c>
@@ -4714,6 +5052,9 @@
       </c>
       <c r="F144" s="2" t="s">
         <v>167</v>
+      </c>
+      <c r="G144" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
@@ -4735,6 +5076,9 @@
       <c r="F145" s="2" t="s">
         <v>183</v>
       </c>
+      <c r="G145" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
@@ -4755,6 +5099,9 @@
       <c r="F146" s="2" t="s">
         <v>185</v>
       </c>
+      <c r="G146" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
@@ -4775,6 +5122,9 @@
       <c r="F147" s="2" t="s">
         <v>187</v>
       </c>
+      <c r="G147" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
@@ -4795,6 +5145,9 @@
       <c r="F148" s="2" t="s">
         <v>167</v>
       </c>
+      <c r="G148" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
@@ -4815,6 +5168,9 @@
       <c r="F149" s="2" t="s">
         <v>179</v>
       </c>
+      <c r="G149" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
@@ -4835,6 +5191,9 @@
       <c r="F150" s="2" t="s">
         <v>167</v>
       </c>
+      <c r="G150" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
@@ -4855,6 +5214,9 @@
       <c r="F151" s="2" t="s">
         <v>181</v>
       </c>
+      <c r="G151" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
@@ -4875,6 +5237,9 @@
       <c r="F152" s="2" t="s">
         <v>280</v>
       </c>
+      <c r="G152" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
@@ -4895,6 +5260,9 @@
       <c r="F153" s="2" t="s">
         <v>278</v>
       </c>
+      <c r="G153" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
@@ -4915,6 +5283,9 @@
       <c r="F154" s="2" t="s">
         <v>282</v>
       </c>
+      <c r="G154" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
@@ -4935,6 +5306,9 @@
       <c r="F155" s="2" t="s">
         <v>276</v>
       </c>
+      <c r="G155" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
@@ -4955,6 +5329,9 @@
       <c r="F156" s="2" t="s">
         <v>87</v>
       </c>
+      <c r="G156" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
@@ -4975,6 +5352,9 @@
       <c r="F157" s="2" t="s">
         <v>75</v>
       </c>
+      <c r="G157" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
@@ -4995,7 +5375,9 @@
       <c r="F158" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G158" s="6"/>
+      <c r="G158" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
@@ -5016,6 +5398,9 @@
       <c r="F159" s="2" t="s">
         <v>81</v>
       </c>
+      <c r="G159" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
@@ -5036,8 +5421,11 @@
       <c r="F160" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G160" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>54</v>
       </c>
@@ -5056,8 +5444,11 @@
       <c r="F161" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G161" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>57</v>
       </c>
@@ -5076,8 +5467,11 @@
       <c r="F162" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G162" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>52</v>
       </c>
@@ -5096,8 +5490,11 @@
       <c r="F163" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G163" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>51</v>
       </c>
@@ -5116,8 +5513,11 @@
       <c r="F164" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G164" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>58</v>
       </c>
@@ -5136,8 +5536,11 @@
       <c r="F165" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G165" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>48</v>
       </c>
@@ -5156,8 +5559,11 @@
       <c r="F166" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G166" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>3</v>
       </c>
@@ -5176,8 +5582,11 @@
       <c r="F167" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G167" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>6</v>
       </c>
@@ -5196,8 +5605,11 @@
       <c r="F168" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G168" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>5</v>
       </c>
@@ -5216,8 +5628,11 @@
       <c r="F169" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G169" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>10</v>
       </c>
@@ -5236,8 +5651,11 @@
       <c r="F170" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G170" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>4</v>
       </c>
@@ -5256,8 +5674,11 @@
       <c r="F171" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G171" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>8</v>
       </c>
@@ -5276,8 +5697,11 @@
       <c r="F172" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G172" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>2</v>
       </c>
@@ -5296,8 +5720,11 @@
       <c r="F173" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G173" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>9</v>
       </c>
@@ -5316,8 +5743,11 @@
       <c r="F174" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G174" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>1</v>
       </c>
@@ -5336,8 +5766,11 @@
       <c r="F175" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G175" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>7</v>
       </c>
@@ -5356,8 +5789,11 @@
       <c r="F176" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G176" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>240</v>
       </c>
@@ -5376,8 +5812,11 @@
       <c r="F177" s="2" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G177" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>237</v>
       </c>
@@ -5396,8 +5835,11 @@
       <c r="F178" s="2" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G178" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
         <v>238</v>
       </c>
@@ -5416,8 +5858,11 @@
       <c r="F179" s="2" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G179" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
         <v>234</v>
       </c>
@@ -5436,8 +5881,11 @@
       <c r="F180" s="2" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G180" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
         <v>230</v>
       </c>
@@ -5456,8 +5904,11 @@
       <c r="F181" s="2" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G181" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
         <v>226</v>
       </c>
@@ -5476,8 +5927,11 @@
       <c r="F182" s="2" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G182" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
         <v>229</v>
       </c>
@@ -5496,8 +5950,11 @@
       <c r="F183" s="2" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G183" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
         <v>233</v>
       </c>
@@ -5516,8 +5973,11 @@
       <c r="F184" s="2" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G184" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
         <v>225</v>
       </c>
@@ -5536,8 +5996,11 @@
       <c r="F185" s="2" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G185" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
         <v>236</v>
       </c>
@@ -5556,8 +6019,11 @@
       <c r="F186" s="2" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G186" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>235</v>
       </c>
@@ -5576,8 +6042,11 @@
       <c r="F187" s="2" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G187" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
         <v>231</v>
       </c>
@@ -5596,8 +6065,11 @@
       <c r="F188" s="2" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G188" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
         <v>244</v>
       </c>
@@ -5616,8 +6088,11 @@
       <c r="F189" s="2" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G189" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
         <v>243</v>
       </c>
@@ -5636,8 +6111,11 @@
       <c r="F190" s="2" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G190" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="2">
         <v>242</v>
       </c>
@@ -5656,8 +6134,11 @@
       <c r="F191" s="2" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G191" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" s="2">
         <v>241</v>
       </c>
@@ -5675,6 +6156,9 @@
       </c>
       <c r="F192" s="2" t="s">
         <v>359</v>
+      </c>
+      <c r="G192" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.25">
@@ -5696,6 +6180,9 @@
       <c r="F193" s="2" t="s">
         <v>335</v>
       </c>
+      <c r="G193" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="2">
@@ -5716,6 +6203,9 @@
       <c r="F194" s="2" t="s">
         <v>337</v>
       </c>
+      <c r="G194" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="2">
@@ -5736,6 +6226,9 @@
       <c r="F195" s="2" t="s">
         <v>343</v>
       </c>
+      <c r="G195" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="2">
@@ -5756,6 +6249,9 @@
       <c r="F196" s="2" t="s">
         <v>355</v>
       </c>
+      <c r="G196" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
@@ -5776,6 +6272,9 @@
       <c r="F197" s="2" t="s">
         <v>385</v>
       </c>
+      <c r="G197" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" s="2">
@@ -5796,7 +6295,9 @@
       <c r="F198" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="G198" s="6"/>
+      <c r="G198" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" s="2">
@@ -5817,7 +6318,9 @@
       <c r="F199" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="G199" s="6"/>
+      <c r="G199" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" s="2">
@@ -5838,6 +6341,9 @@
       <c r="F200" s="2" t="s">
         <v>389</v>
       </c>
+      <c r="G200" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" s="2">
@@ -5858,6 +6364,9 @@
       <c r="F201" s="2" t="s">
         <v>391</v>
       </c>
+      <c r="G201" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" s="2">
@@ -5878,6 +6387,9 @@
       <c r="F202" s="2" t="s">
         <v>393</v>
       </c>
+      <c r="G202" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" s="2">
@@ -5898,6 +6410,9 @@
       <c r="F203" s="2" t="s">
         <v>395</v>
       </c>
+      <c r="G203" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" s="2">
@@ -5918,6 +6433,9 @@
       <c r="F204" s="2" t="s">
         <v>397</v>
       </c>
+      <c r="G204" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="2">
@@ -5938,6 +6456,9 @@
       <c r="F205" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="G205" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="2">
@@ -5958,6 +6479,9 @@
       <c r="F206" s="2" t="s">
         <v>399</v>
       </c>
+      <c r="G206" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="2">
@@ -5978,6 +6502,9 @@
       <c r="F207" s="2" t="s">
         <v>401</v>
       </c>
+      <c r="G207" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="2">
@@ -5998,8 +6525,11 @@
       <c r="F208" s="2" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G208" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" s="2">
         <v>663</v>
       </c>
@@ -6018,8 +6548,11 @@
       <c r="F209" s="2" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G209" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="2">
         <v>661</v>
       </c>
@@ -6038,8 +6571,11 @@
       <c r="F210" s="2" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G210" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="2">
         <v>662</v>
       </c>
@@ -6058,8 +6594,11 @@
       <c r="F211" s="2" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G211" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" s="2">
         <v>46</v>
       </c>
@@ -6078,8 +6617,11 @@
       <c r="F212" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G212" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" s="2">
         <v>32</v>
       </c>
@@ -6098,8 +6640,11 @@
       <c r="F213" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G213" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="2">
         <v>21</v>
       </c>
@@ -6118,8 +6663,11 @@
       <c r="F214" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G214" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" s="2">
         <v>35</v>
       </c>
@@ -6138,8 +6686,11 @@
       <c r="F215" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G215" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="2">
         <v>24</v>
       </c>
@@ -6158,8 +6709,11 @@
       <c r="F216" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G216" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="2">
         <v>19</v>
       </c>
@@ -6178,8 +6732,11 @@
       <c r="F217" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G217" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="2">
         <v>26</v>
       </c>
@@ -6198,8 +6755,11 @@
       <c r="F218" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G218" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="2">
         <v>14</v>
       </c>
@@ -6218,8 +6778,11 @@
       <c r="F219" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G219" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="2">
         <v>12</v>
       </c>
@@ -6238,8 +6801,11 @@
       <c r="F220" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G220" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="2">
         <v>11</v>
       </c>
@@ -6258,8 +6824,11 @@
       <c r="F221" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G221" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" s="2">
         <v>33</v>
       </c>
@@ -6278,8 +6847,11 @@
       <c r="F222" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G222" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="2">
         <v>16</v>
       </c>
@@ -6298,8 +6870,11 @@
       <c r="F223" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G223" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" s="2">
         <v>28</v>
       </c>
@@ -6318,8 +6893,11 @@
       <c r="F224" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G224" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" s="2">
         <v>18</v>
       </c>
@@ -6338,8 +6916,11 @@
       <c r="F225" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G225" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" s="2">
         <v>31</v>
       </c>
@@ -6358,8 +6939,11 @@
       <c r="F226" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G226" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" s="2">
         <v>34</v>
       </c>
@@ -6378,8 +6962,11 @@
       <c r="F227" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G227" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" s="2">
         <v>27</v>
       </c>
@@ -6398,8 +6985,11 @@
       <c r="F228" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G228" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" s="2">
         <v>17</v>
       </c>
@@ -6418,8 +7008,11 @@
       <c r="F229" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G229" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230" s="2">
         <v>29</v>
       </c>
@@ -6438,8 +7031,11 @@
       <c r="F230" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G230" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231" s="2">
         <v>15</v>
       </c>
@@ -6458,8 +7054,11 @@
       <c r="F231" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G231" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232" s="2">
         <v>13</v>
       </c>
@@ -6478,8 +7077,11 @@
       <c r="F232" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G232" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" s="2">
         <v>30</v>
       </c>
@@ -6498,8 +7100,11 @@
       <c r="F233" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G233" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234" s="2">
         <v>36</v>
       </c>
@@ -6518,8 +7123,11 @@
       <c r="F234" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G234" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" s="2">
         <v>25</v>
       </c>
@@ -6538,8 +7146,11 @@
       <c r="F235" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G235" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236" s="2">
         <v>41</v>
       </c>
@@ -6558,8 +7169,11 @@
       <c r="F236" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G236" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" s="2">
         <v>20</v>
       </c>
@@ -6578,8 +7192,11 @@
       <c r="F237" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G237" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" s="2">
         <v>37</v>
       </c>
@@ -6598,8 +7215,11 @@
       <c r="F238" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G238" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239" s="2">
         <v>39</v>
       </c>
@@ -6618,8 +7238,11 @@
       <c r="F239" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G239" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240" s="2">
         <v>45</v>
       </c>
@@ -6637,6 +7260,9 @@
       </c>
       <c r="F240" s="2" t="s">
         <v>65</v>
+      </c>
+      <c r="G240" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.25">
@@ -6658,6 +7284,9 @@
       <c r="F241" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="G241" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242" s="2">
@@ -6678,6 +7307,9 @@
       <c r="F242" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="G242" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243" s="2">
@@ -6698,6 +7330,9 @@
       <c r="F243" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="G243" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244" s="2">
@@ -6718,6 +7353,9 @@
       <c r="F244" s="2" t="s">
         <v>63</v>
       </c>
+      <c r="G244" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="245" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A245" s="2">
@@ -6738,6 +7376,9 @@
       <c r="F245" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="G245" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="246" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A246" s="2">
@@ -6758,7 +7399,9 @@
       <c r="F246" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G246" s="6"/>
+      <c r="G246" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247" s="2">
@@ -6779,7 +7422,9 @@
       <c r="F247" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G247" s="6"/>
+      <c r="G247" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248" s="2">
@@ -6800,7 +7445,9 @@
       <c r="F248" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G248" s="6"/>
+      <c r="G248" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A249" s="2">
@@ -6817,6 +7464,9 @@
       </c>
       <c r="E249" s="2"/>
       <c r="F249" s="2"/>
+      <c r="G249" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250" s="2">
@@ -6833,7 +7483,9 @@
       </c>
       <c r="E250" s="2"/>
       <c r="F250" s="2"/>
-      <c r="G250" s="6"/>
+      <c r="G250" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251" s="2">
@@ -6850,6 +7502,9 @@
       </c>
       <c r="E251" s="2"/>
       <c r="F251" s="2"/>
+      <c r="G251" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A252" s="2">
@@ -6866,6 +7521,9 @@
       </c>
       <c r="E252" s="2"/>
       <c r="F252" s="2"/>
+      <c r="G252" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253" s="2">
@@ -6882,6 +7540,9 @@
       </c>
       <c r="E253" s="2"/>
       <c r="F253" s="2"/>
+      <c r="G253" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="254" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A254" s="2">
@@ -6898,6 +7559,9 @@
       </c>
       <c r="E254" s="2"/>
       <c r="F254" s="2"/>
+      <c r="G254" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" s="2">
@@ -6914,6 +7578,9 @@
       </c>
       <c r="E255" s="2"/>
       <c r="F255" s="2"/>
+      <c r="G255" s="5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A256" s="2">
@@ -6930,8 +7597,11 @@
       </c>
       <c r="E256" s="2"/>
       <c r="F256" s="2"/>
-    </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G256" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A257" s="2">
         <v>2607</v>
       </c>
@@ -6946,8 +7616,11 @@
       </c>
       <c r="E257" s="2"/>
       <c r="F257" s="2"/>
-    </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G257" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A258" s="2">
         <v>2611</v>
       </c>
@@ -6962,8 +7635,11 @@
       </c>
       <c r="E258" s="2"/>
       <c r="F258" s="2"/>
-    </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G258" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A259" s="2">
         <v>2618</v>
       </c>
@@ -6978,8 +7654,11 @@
       </c>
       <c r="E259" s="2"/>
       <c r="F259" s="2"/>
-    </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G259" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A260" s="2">
         <v>2619</v>
       </c>
@@ -6994,8 +7673,11 @@
       </c>
       <c r="E260" s="2"/>
       <c r="F260" s="2"/>
-    </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G260" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A261" s="2">
         <v>2612</v>
       </c>
@@ -7010,8 +7692,11 @@
       </c>
       <c r="E261" s="2"/>
       <c r="F261" s="2"/>
-    </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G261" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A262" s="2">
         <v>2608</v>
       </c>
@@ -7026,8 +7711,11 @@
       </c>
       <c r="E262" s="2"/>
       <c r="F262" s="2"/>
-    </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G262" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A263" s="2">
         <v>2609</v>
       </c>
@@ -7042,8 +7730,11 @@
       </c>
       <c r="E263" s="2"/>
       <c r="F263" s="2"/>
-    </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G263" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A264" s="2">
         <v>2621</v>
       </c>
@@ -7058,8 +7749,11 @@
       </c>
       <c r="E264" s="2"/>
       <c r="F264" s="2"/>
-    </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G264" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A265" s="2">
         <v>2613</v>
       </c>
@@ -7074,8 +7768,11 @@
       </c>
       <c r="E265" s="2"/>
       <c r="F265" s="2"/>
-    </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G265" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A266" s="2">
         <v>2614</v>
       </c>
@@ -7090,8 +7787,11 @@
       </c>
       <c r="E266" s="2"/>
       <c r="F266" s="2"/>
-    </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G266" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A267" s="2">
         <v>2615</v>
       </c>
@@ -7106,8 +7806,11 @@
       </c>
       <c r="E267" s="2"/>
       <c r="F267" s="2"/>
-    </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G267" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A268" s="2">
         <v>2610</v>
       </c>
@@ -7122,8 +7825,11 @@
       </c>
       <c r="E268" s="2"/>
       <c r="F268" s="2"/>
-    </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G268" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A269" s="2">
         <v>2620</v>
       </c>
@@ -7138,8 +7844,11 @@
       </c>
       <c r="E269" s="2"/>
       <c r="F269" s="2"/>
-    </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G269" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A270" s="2">
         <v>259</v>
       </c>
@@ -7154,8 +7863,11 @@
       </c>
       <c r="E270" s="2"/>
       <c r="F270" s="2"/>
-    </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G270" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A271" s="2">
         <v>251</v>
       </c>
@@ -7174,8 +7886,11 @@
       <c r="F271" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G271" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A272" s="2">
         <v>255</v>
       </c>
@@ -7194,8 +7909,11 @@
       <c r="F272" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G272" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A273" s="2">
         <v>253</v>
       </c>
@@ -7214,8 +7932,11 @@
       <c r="F273" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G273" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A274" s="2">
         <v>246</v>
       </c>
@@ -7234,8 +7955,11 @@
       <c r="F274" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G274" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A275" s="2">
         <v>248</v>
       </c>
@@ -7254,8 +7978,11 @@
       <c r="F275" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G275" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A276" s="2">
         <v>247</v>
       </c>
@@ -7274,8 +8001,11 @@
       <c r="F276" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G276" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A277" s="2">
         <v>252</v>
       </c>
@@ -7294,8 +8024,11 @@
       <c r="F277" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G277" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A278" s="2">
         <v>256</v>
       </c>
@@ -7314,8 +8047,11 @@
       <c r="F278" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G278" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A279" s="2">
         <v>250</v>
       </c>
@@ -7334,8 +8070,11 @@
       <c r="F279" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G279" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A280" s="2">
         <v>257</v>
       </c>
@@ -7354,8 +8093,11 @@
       <c r="F280" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G280" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A281" s="2">
         <v>258</v>
       </c>
@@ -7374,8 +8116,11 @@
       <c r="F281" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G281" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A282" s="2">
         <v>254</v>
       </c>
@@ -7394,8 +8139,11 @@
       <c r="F282" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G282" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A283" s="2">
         <v>249</v>
       </c>
@@ -7414,8 +8162,11 @@
       <c r="F283" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G283" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A284" s="2">
         <v>245</v>
       </c>
@@ -7433,6 +8184,9 @@
       </c>
       <c r="F284" s="2" t="s">
         <v>366</v>
+      </c>
+      <c r="G284" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>